<commit_message>
feat(note): display NOTE column (e.g. frequency) inside node boxes
- Add 'note' field to Node dataclass
- Parse NOTE column in parser.py (optional, backward compatible)
- Show note below node name in both drawio and excalidraw renderers
- Regenerate all example outputs
</commit_message>
<xml_diff>
--- a/crg_drawio/input/clock_table.xlsx
+++ b/crg_drawio/input/clock_table.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClockTree" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,7 +459,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>OCC/SCAN MUX</t>
+          <t>OCC</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -483,11 +483,6 @@
         </is>
       </c>
       <c r="N1" t="inlineStr">
-        <is>
-          <t>CE_DISEN</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
         <is>
           <t>ATTR</t>
         </is>
@@ -511,8 +506,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>input</t>
         </is>
@@ -536,8 +530,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>input</t>
         </is>
@@ -561,8 +554,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>input</t>
         </is>
@@ -586,8 +578,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>input</t>
         </is>
@@ -611,8 +602,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>input</t>
         </is>
@@ -636,8 +626,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>internal</t>
         </is>
@@ -662,7 +651,6 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -694,8 +682,7 @@
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -731,8 +718,7 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -768,8 +754,7 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -797,8 +782,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -834,8 +818,7 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -883,8 +866,7 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -920,8 +902,7 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -957,8 +938,7 @@
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -994,8 +974,7 @@
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1031,8 +1010,7 @@
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1068,8 +1046,7 @@
           <t>pmu_mcu_clkgate_req</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>internal</t>
         </is>
@@ -1109,8 +1086,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1138,8 +1114,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1167,8 +1142,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>internal</t>
         </is>
@@ -1216,8 +1190,7 @@
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1253,8 +1226,7 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1294,8 +1266,7 @@
           <t>pmu_main_clkgate_req</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1343,8 +1314,7 @@
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1376,8 +1346,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1425,8 +1394,7 @@
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>output</t>
         </is>
@@ -1474,8 +1442,7 @@
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>output</t>
         </is>

</xml_diff>